<commit_message>
docs: update BANG_MA_LOI_HE_THONG.xlsx with dynamic debounce and full event logging logic sheet
</commit_message>
<xml_diff>
--- a/docs/BANG_MA_LOI_HE_THONG.xlsx
+++ b/docs/BANG_MA_LOI_HE_THONG.xlsx
@@ -8,6 +8,7 @@
   <sheets>
     <sheet name="Danh mục mã lỗi" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Cấp độ hành vi xử lý" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Logic ghi nhật ký (Log)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh mục mã lỗi'!$A$1:$G$39</definedName>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,6 +53,33 @@
       <b val="1"/>
       <color rgb="00800000"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="7">
@@ -117,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -160,6 +188,23 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -566,13 +611,13 @@
   <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="85" customWidth="1" min="7" max="7"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="65" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -635,7 +680,7 @@
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>Cảnh báo (INFO)</t>
+          <t>Dừng sạc an toàn (STOP) (Bypass ở PRECHARGE)</t>
         </is>
       </c>
       <c r="F2" s="8" t="inlineStr">
@@ -645,7 +690,7 @@
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>Nhận bản tin ALM_INFO (0x07F4), trường low_pack_volt với severity &gt;= 2. ev_bms() kiểm tra (in-&gt;bms.alarm_flags &amp; BMS_ALARM_LOW_PACK_VOLT) != 0.</t>
+          <t>Nhận bản tin ALM_INFO (0x07F4), trường low_pack_volt với severity &gt;= 1, HOẶC ở chế độ BMS_CONTROLLED (ngoài PRECHARGE) đo được 0.5*Vmax &lt;= Vbatt &lt; Vmin. Tự động bypass trong PRECHARGE.</t>
         </is>
       </c>
     </row>
@@ -783,7 +828,7 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Dừng sạc an toàn (STOP)</t>
+          <t>Tự phục hồi tối đa 3 lần, lần 4 Dừng sạc (STOP)</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -793,7 +838,7 @@
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Nhận bản tin ALM_INFO (0x07F4), trường temp_cell_high_chg với severity &gt;= 2. ev_bms() kiểm tra (in-&gt;bms.alarm_flags &amp; BMS_ALARM_TEMP_HIGH_CHG) != 0.</t>
+          <t>Nhận bản tin ALM_INFO (0x07F4) trường temp_cell_high_chg HOẶC max_cell_temp &gt;= temp_limit_c. Kẹp dòng 0A (inhibit=1), tự phục hồi tối đa 3 lần sau 3s làm mát ổn định. Quá nhiệt lần 4 chuyển FAULT dừng hẳn.</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1171,7 @@
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>Bộ sạc tự phát hiện và gửi qua CAN (Mirror 1:1): Kiểm tra trực tiếp cờ (in-&gt;mod_alarm_or &amp; CHG_LIB_ALARM_HW_FAULT) != 0.</t>
+          <t>Nhận cờ CAN từ bộ sạc: (in-&gt;mod_alarm_or &amp; CHG_LIB_ALARM_HW_FAULT) != 0. Debounce động theo trạng thái: IDLE = 10.000ms (10s) để lọc sạch xung xả tụ/sụt áp khi ngắt Aptomat AC; ACTIVE/RUNNING = 1.000ms (1s) ngắt sạc nhanh an toàn. Tự động suppress khi có sụt áp AC, lỗi PFC, mất pha lưới hoặc khi module offline trong IDLE.</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1393,7 @@
       </c>
       <c r="G21" s="12" t="inlineStr">
         <is>
-          <t>Bộ sạc tự phát hiện và gửi qua CAN (Mirror 1:1): ev_mod_pfc kiểm tra cờ PFC fault từ bộ sạc.</t>
+          <t>Nhận cờ CAN lỗi PFC/mất pha từ bộ sạc: ev_mod_pfc kích hoạt. Tự động bypass ở IDLE (chống báo ảo khi ngắt AC), suppress khi có cờ thấp áp AC.</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1504,7 @@
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>Bộ sạc tự phát hiện và gửi qua CAN (Mirror 1:1): Kiểm tra trực tiếp cờ (in-&gt;mod_alarm_or &amp; CHG_LIB_ALARM_AC_UNDER_VOLT) != 0. Debounce lọc 5000ms để chống báo ảo do tụ nguồn DC-bus xả điện khi ngắt nguồn AC / dập aptomat.</t>
+          <t>Nhận cờ CAN thấp áp AC: (in-&gt;mod_alarm_or &amp; CHG_LIB_ALARM_AC_UNDER_VOLT) != 0. Tự động bypass trong IDLE (Clean Shutdown); trong active session debounce set 1000ms, clear 3000ms.</t>
         </is>
       </c>
     </row>
@@ -1774,10 +1819,10 @@
   <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12.875" customWidth="1" min="1" max="1"/>
-    <col width="22.875" customWidth="1" min="2" max="2"/>
-    <col width="35.875" customWidth="1" min="3" max="3"/>
-    <col width="80.875" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -1848,9 +1893,9 @@
         <is>
           <t>1. Gọi ChargeController_Stop(reason).
 2. Gửi lệnh giảm dòng mục tiêu target_current = 0A qua mạng CAN tới tất cả module.
-3. Chờ dòng điện phản hồi thực tế giảm xuống &lt; 2.0A (ALARM_I_LOAD_MIN_A) để dập hồ quang.
+3. Chờ dòng điện phản hồi thực tế giảm xuống &lt; 1.0A (RELAY_OPEN_CURRENT_THRESHOLD_A) để dập hồ quang (hoặc timeout 3000ms).
 4. Mở rơ-le / contactor DC ngõ ra sạc.
-5. Ghi log sự kiện vào vòng đệm AlarmLogEntry_t (sâu 24 bản ghi).</t>
+5. Ghi log sự kiện vào RAM Ring Buffer (sâu 16 bản ghi) và lưu trữ vĩnh viễn vào External SPI Flash (W25Qxx).</t>
         </is>
       </c>
     </row>
@@ -1907,4 +1952,780 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="65" customWidth="1" min="1" max="1"/>
+    <col width="41" customWidth="1" min="2" max="2"/>
+    <col width="63" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="4" max="4"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
+    <col width="65" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>KIẾN TRÚC VÀ LOGIC GHI NHẬT KÝ LỖI (ALARM &amp; EVENT LOGGING)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>1. Cấu trúc Bộ đệm &amp; Vòng đời Bản ghi Log</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Thành phần</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>Vị trí phần cứng</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>Độ sâu / Quy mô</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>Mục đích sử dụng</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>Cơ chế hoạt động</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>RAM Ring Buffer</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>SRAM vi điều khiển (STM32)</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>16 bản ghi mới nhất</t>
+        </is>
+      </c>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>Hiển thị tức thời trên HMI DWIN (Trang 10 - Nhật ký lỗi)</t>
+        </is>
+      </c>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>Bộ đệm vòng FIFO (g_alarm.log). Ghi đè bản ghi cũ nhất khi đầy. Mất dữ liệu khi mất nguồn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>External SPI Flash</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Chip nhớ W25Qxx trên bo mạch</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>Phân vùng Flash không bay hơi</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>Lưu trữ vĩnh viễn, truy xuất bảo hành và kiểm toán</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>Hàm AlarmStorage_Append() ghi trực tiếp ngay khi có sự kiện. Không mất dữ liệu khi tắt nguồn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Cổng giao tiếp PC</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>UART / USB Debug Protocol</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>Toàn bộ lịch sử Flash</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>Tải lịch sử sự cố ra file CSV trên máy tính</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>Lệnh nhị phân CMD_GET_ALARM_LOG cho phép PC App đọc toàn bộ bản ghi phục vụ phân tích.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Giới hạn Console</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>UART Console / RTT Terminal</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>1000ms (1s rate limit)</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Bảo vệ timing ngắt và chống nghẽn đường truyền UART</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>ALARM_LOG_MIN_INTERVAL_MS gom các sự kiện trong tick để xuất 1 dòng tóm tắt duy nhất.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>2. Định dạng Cấu trúc Bản ghi Sự kiện (AlarmLogEntry_t - 8 Bytes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Trường dữ liệu</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Kiểu dữ liệu</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>Kích thước</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>Ý nghĩa &amp; Dải giá trị</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>Mô tả chi tiết</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>uptime_ms</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>uint32_t</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>4 bytes</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>0 .. 4.294.967.295 ms</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>Thời gian hệ thống (Tick Uptime) tính từ lúc cấp nguồn trạm sạc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>uint16_t</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>2 bytes</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>0 .. 65535 (AlarmCode_t)</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>Mã định danh lỗi: ánh xạ trực tiếp sang E001..E032, W001..W011.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>uint8_t</t>
+        </is>
+      </c>
+      <c r="C14" s="20" t="inlineStr">
+        <is>
+          <t>1 byte</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>0=NONE, 1=INFO, 2=STOP, 3=ESTOP</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>Cấp hành vi xử lý an toàn tương ứng với mã lỗi khi xuất hiện.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>uint8_t</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>1 byte</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>1 = RAISED, 0 = CLEARED</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>Sườn chuyển đổi: 1 là thời điểm lỗi bắt đầu xuất hiện; 0 là thời điểm lỗi tự xóa/hết.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>timestamp (phụ)</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>uint32_t</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>4 bytes</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>Unix Epoch (giây kể từ 1970)</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>Thời gian thực lấy từ chip RTC ngoại (DS3231/STM32 RTC). Trả về 0 nếu RTC chưa đồng bộ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>3. Bảng Cấu hình Debounce Động theo Trạng thái Vận hành (Dynamic Debounce)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Mã lỗi</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>Tên lỗi</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>Debounce IDLE (Chờ)</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>Debounce ACTIVE (Đang sạc)</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>Clear Debounce</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="inlineStr">
+        <is>
+          <t>Lý do thiết kế &amp; Ý nghĩa an toàn</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>E010</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>Lỗi phần cứng module (HW Fault)</t>
+        </is>
+      </c>
+      <c r="C20" s="20" t="inlineStr">
+        <is>
+          <t>10.000 ms (10 giây)</t>
+        </is>
+      </c>
+      <c r="D20" s="20" t="inlineStr">
+        <is>
+          <t>1.000 ms (1 giây)</t>
+        </is>
+      </c>
+      <c r="E20" s="20" t="inlineStr">
+        <is>
+          <t>200 ms</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>Ở IDLE: Nuốt trọn 100% xung xả tụ và sụt áp DC-bus khi ngắt Aptomat AC (kéo dài 200ms-1.5s), loại bỏ báo giả E010. Khi ACTIVE: Phản ứng ngắt sạc nhanh 1s. Bắt lỗi tĩnh IDLE sau 10s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>W011</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>Điện lưới AC yếu / mất pha</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>Bypass (Không bắt lỗi)</t>
+        </is>
+      </c>
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>1.000 ms (1 giây)</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="inlineStr">
+        <is>
+          <t>3.000 ms</t>
+        </is>
+      </c>
+      <c r="F21" s="19" t="inlineStr">
+        <is>
+          <t>Ở IDLE: Ngắt AC là hành vi tắt trạm bình thường (Clean Shutdown), không sinh cảnh báo. Khi ACTIVE: Cảnh báo sau 1s nếu điện lưới sụt dưới ngưỡng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>E015</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>Lỗi khối nguồn PFC</t>
+        </is>
+      </c>
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>Bypass (Không bắt lỗi)</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>0 ms (Tức thì)</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>200 ms</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr">
+        <is>
+          <t>Ở IDLE: Bypass tránh báo lỗi khi ngắt AC. Khi sạc: Ngắt ngay lập tức bảo vệ tầng chỉnh lưu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>W010</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>Mất giao tiếp CAN module</t>
+        </is>
+      </c>
+      <c r="C23" s="20" t="inlineStr">
+        <is>
+          <t>Bypass (Không bắt lỗi)</t>
+        </is>
+      </c>
+      <c r="D23" s="20" t="inlineStr">
+        <is>
+          <t>2.000 ms (2 giây)</t>
+        </is>
+      </c>
+      <c r="E23" s="20" t="inlineStr">
+        <is>
+          <t>200 ms</t>
+        </is>
+      </c>
+      <c r="F23" s="19" t="inlineStr">
+        <is>
+          <t>Ở IDLE: Tránh báo mất kết nối khi trạm đang tắt nguồn. Khi sạc: Cảnh báo/dừng sau 2s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>E023</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>Mất tải DC đột ngột</t>
+        </is>
+      </c>
+      <c r="C24" s="20" t="inlineStr">
+        <is>
+          <t>Không kích hoạt ở IDLE</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>800 ms</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>Chốt (Latching)</t>
+        </is>
+      </c>
+      <c r="F24" s="19" t="inlineStr">
+        <is>
+          <t>Chỉ đánh giá khi RUNNING có dòng sạc. Nhận diện rút súng sạc đột ngột (Hot Unplug) khi dòng tụt &lt;15% mà áp vẫn &gt;98%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>E012/E013</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>Quá áp DC / Ngắn mạch đầu ra</t>
+        </is>
+      </c>
+      <c r="C25" s="20" t="inlineStr">
+        <is>
+          <t>0 ms (ESTOP tức thì)</t>
+        </is>
+      </c>
+      <c r="D25" s="20" t="inlineStr">
+        <is>
+          <t>0 ms (ESTOP tức thì)</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="inlineStr">
+        <is>
+          <t>200 ms</t>
+        </is>
+      </c>
+      <c r="F25" s="19" t="inlineStr">
+        <is>
+          <t>Lỗi an toàn cháy nổ khẩn cấp: Ngắt xung module và mở relay ngay lập tức ở mọi trạng thái.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>E011/E014</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>Quá nhiệt / Quá dòng module</t>
+        </is>
+      </c>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>0 ms (STOP tức thì)</t>
+        </is>
+      </c>
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>0 ms (STOP tức thì)</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="inlineStr">
+        <is>
+          <t>200 ms</t>
+        </is>
+      </c>
+      <c r="F26" s="19" t="inlineStr">
+        <is>
+          <t>Bảo vệ phần cứng công suất tức thì, không áp dụng trễ lọc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>4. Ma trận Chế áp Lỗi Dây chuyền (Cascade Suppression Matrix)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>Sự kiện gốc (Root Cause)</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>Lỗi gốc được ghi nhận</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>Các lỗi phái sinh bị CHẾ ÁP (Suppressed)</t>
+        </is>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
+        <is>
+          <t>Cơ chế cô lập trong Firmware</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>Mục tiêu chất lượng Log</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>Ngắt Aptomat AC / Mất điện lưới lúc IDLE</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="inlineStr">
+        <is>
+          <t>Không ghi lỗi (Clean Shutdown)</t>
+        </is>
+      </c>
+      <c r="C30" s="20" t="inlineStr">
+        <is>
+          <t>E010, E015, W010, W011</t>
+        </is>
+      </c>
+      <c r="D30" s="19" t="inlineStr">
+        <is>
+          <t>Hàm eval kiểm tra in-&gt;cc.state == IDLE và in-&gt;mod_offline_count != 0 -&gt; trả về false; kết hợp debounce 10s nuốt trọn xả tụ.</t>
+        </is>
+      </c>
+      <c r="E30" s="19" t="inlineStr">
+        <is>
+          <t>Triệt tiêu 100% log rác và cảnh báo giả khi tắt nguồn trạm sạc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="inlineStr">
+        <is>
+          <t>Mất điện lưới AC / Sụt áp AC khi đang sạc</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="inlineStr">
+        <is>
+          <t>W011 (hoặc dừng an toàn)</t>
+        </is>
+      </c>
+      <c r="C31" s="20" t="inlineStr">
+        <is>
+          <t>E010 (Lỗi HW), E015 (Lỗi PFC), W010 (Mất CAN)</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="inlineStr">
+        <is>
+          <t>Khi có cờ AC_UNDER_VOLT hoặc W011 active, ev_mod_hw_fault() và ev_mod_pfc() tự động suppress E010 và E015.</t>
+        </is>
+      </c>
+      <c r="E31" s="19" t="inlineStr">
+        <is>
+          <t>Chỉ ghi nhận đúng nguyên nhân gốc là do điện lưới, không đổ lỗi cho phần cứng bộ sạc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr">
+        <is>
+          <t>Rút giắc sạc đột ngột (Hot Unplug) khi đang sạc</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="inlineStr">
+        <is>
+          <t>E023 (Mất tải DC đột ngột)</t>
+        </is>
+      </c>
+      <c r="C32" s="20" t="inlineStr">
+        <is>
+          <t>E021 (Mất CAN pin), E022 (Không có pin)</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="inlineStr">
+        <is>
+          <t>ev_bms_comm_lost() và ev_bms_no_pack_voltage() kiểm tra is_alarm_active_or_latched(ALARM_DC_LOAD_LOST) -&gt; suppress hoàn toàn.</t>
+        </is>
+      </c>
+      <c r="E32" s="19" t="inlineStr">
+        <is>
+          <t>Ngăn chặn hiện tượng giật giắc sạc gây bão 3-4 mã lỗi đồng thời.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="18" t="inlineStr">
+        <is>
+          <t>Bảo vệ ngắt quá nhiệt khối pin (Thermal Pause)</t>
+        </is>
+      </c>
+      <c r="B33" s="20" t="inlineStr">
+        <is>
+          <t>E005 (Cảnh báo quá nhiệt, kẹp dòng 0A)</t>
+        </is>
+      </c>
+      <c r="C33" s="20" t="inlineStr">
+        <is>
+          <t>E023 (Mất tải DC), E024 (Chưa có đầu ra), E030 (Sụt áp jack)</t>
+        </is>
+      </c>
+      <c r="D33" s="19" t="inlineStr">
+        <is>
+          <t>ev_dc_load_lost() và ev_dc_out_not_established() kiểm tra in-&gt;cc.inhibit != 0 và cờ bms_thermal_alarm -&gt; suppress.</t>
+        </is>
+      </c>
+      <c r="E33" s="19" t="inlineStr">
+        <is>
+          <t>Tránh hiểu nhầm việc chủ động dừng dòng để làm mát pin là sự cố mất tải đường dây.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="18" t="inlineStr">
+        <is>
+          <t>Lỗi bảo vệ phần cứng module cụ thể</t>
+        </is>
+      </c>
+      <c r="B34" s="20" t="inlineStr">
+        <is>
+          <t>E011, E012, E013, E014, E016, E017</t>
+        </is>
+      </c>
+      <c r="C34" s="20" t="inlineStr">
+        <is>
+          <t>E010 (Lỗi phần cứng chung)</t>
+        </is>
+      </c>
+      <c r="D34" s="19" t="inlineStr">
+        <is>
+          <t>ev_mod_hw_fault() loại trừ specific_mask (nhiệt, áp, dòng, quạt, ngắn mạch), chỉ kích hoạt khi không có mã cụ thể nào.</t>
+        </is>
+      </c>
+      <c r="E34" s="19" t="inlineStr">
+        <is>
+          <t>Phân định chính xác hỏng hóc ở bộ phận nào, không ghi đè mã chung chung E010.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add exact numerical thresholds and timings column to error code excel and markdown
</commit_message>
<xml_diff>
--- a/docs/BANG_MA_LOI_HE_THONG.xlsx
+++ b/docs/BANG_MA_LOI_HE_THONG.xlsx
@@ -145,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -205,6 +205,12 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -608,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -618,6 +624,7 @@
     <col width="62" customWidth="1" min="5" max="5"/>
     <col width="65" customWidth="1" min="6" max="6"/>
     <col width="65" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -656,6 +663,11 @@
           <t>Logic phát hiện trong Code (Không suy diễn)</t>
         </is>
       </c>
+      <c r="H1" s="22" t="inlineStr">
+        <is>
+          <t>Thông số kỹ thuật &amp; Ngưỡng kích hoạt cụ thể (Thresholds &amp; Timings)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
@@ -693,6 +705,14 @@
           <t>Nhận bản tin ALM_INFO (0x07F4), trường low_pack_volt với severity &gt;= 1, HOẶC ở chế độ BMS_CONTROLLED (ngoài PRECHARGE) đo được 0.5*Vmax &lt;= Vbatt &lt; Vmin. Tự động bypass trong PRECHARGE.</t>
         </is>
       </c>
+      <c r="H2" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng điện áp: 0.5 * Vmax &lt;= Vbatt &lt; Vmin (Vmax, Vmin từ cấu hình sạc).
+• Ví dụ hệ pin 72V (Vmax=84V, Vmin=60V): 42V &lt;= Vbatt &lt; 60V kích hoạt lỗi.
+• Debounce set: 0ms, clear: 200ms.
+• Tự động BYPASS hoàn toàn khi trạm ở chế độ PRECHARGE.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="11" t="inlineStr">
@@ -730,6 +750,13 @@
           <t>Nhận bản tin ALM_INFO (0x07F4), trường low_cell_volt với severity &gt;= 2. ev_bms() kiểm tra (in-&gt;bms.alarm_flags &amp; BMS_ALARM_LOW_CELL_VOLT) != 0.</t>
         </is>
       </c>
+      <c r="H3" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng điện áp cell: V_cell &lt; 2.5V (Pin LFP) hoặc &lt; 3.0V (Pin NMC).
+• Kích hoạt theo cờ low_cell_volt severity &gt;= 1 từ bản tin ALM_INFO.
+• Debounce set: 0ms, clear: 200ms.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
@@ -767,6 +794,14 @@
           <t>Nhận bản tin ALM_INFO (0x07F4), trường high_pack_volt với severity &gt;= 2. ev_bms() kiểm tra (in-&gt;bms.alarm_flags &amp; BMS_ALARM_HIGH_PACK_VOLT) != 0.</t>
         </is>
       </c>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng quá áp pack: Vbatt &gt;= Vmax (hoặc Vbatt &gt;= V_bms_ovp).
+• Ví dụ hệ pin 72V (Vmax=84V): Vbatt &gt;= 84.0V.
+• Cờ high_pack_volt từ BMS.
+• Debounce set: 0ms, ngắt STOP tức thì.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
@@ -804,6 +839,13 @@
           <t>Nhận bản tin ALM_INFO (0x07F4), trường high_cell_volt với severity &gt;= 2. ev_bms() kiểm tra (in-&gt;bms.alarm_flags &amp; BMS_ALARM_HIGH_CELL_VOLT) != 0.</t>
         </is>
       </c>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng quá áp cell: V_cell &gt;= 3.65V (Pin LFP) hoặc &gt;= 4.25V (Pin NMC).
+• Cờ high_cell_volt từ bản tin ALM_INFO.
+• Debounce set: 0ms, ngắt STOP tức thì.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
@@ -841,6 +883,14 @@
           <t>Nhận bản tin ALM_INFO (0x07F4) trường temp_cell_high_chg HOẶC max_cell_temp &gt;= temp_limit_c. Kẹp dòng 0A (inhibit=1), tự phục hồi tối đa 3 lần sau 3s làm mát ổn định. Quá nhiệt lần 4 chuyển FAULT dừng hẳn.</t>
         </is>
       </c>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng ngắt quá nhiệt: T_cell &gt;= Temp Limit (mặc định 55°C, dải cấu hình 45°C - 65°C) HOẶC chạm tầng 5 temp_5_c.
+• Hysteresis làm mát: T_cell &lt;= (Temp Limit - 5°C) (temp_delta_c = 5°C).
+• Thời gian làm mát giữ ổn định: &gt;= 3.0 giây.
+• Kẹp dòng 0A tối đa 3 lần; lần thứ 4 khóa chuyển FAULT ngắt hẳn.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
@@ -878,6 +928,13 @@
           <t>Nhận bản tin ALM_INFO (0x07F4), trường temp_cell_low_chg với severity &gt;= 2. ev_bms() kiểm tra (in-&gt;bms.alarm_flags &amp; BMS_ALARM_TEMP_LOW_CHG) != 0.</t>
         </is>
       </c>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng nhiệt độ thấp: T_cell &lt; 0°C.
+• Cờ temp_cell_low_chg từ BMS.
+• Debounce set: 0ms, ngắt STOP bảo vệ mạ lithium.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -915,6 +972,13 @@
           <t>Nhận bản tin ALM_INFO (0x07F4), trường over_chg_curr với severity &gt;= 2. ev_bms() kiểm tra (in-&gt;bms.alarm_flags &amp; BMS_ALARM_OVER_CHG_CURR) != 0.</t>
         </is>
       </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng quá dòng sạc: I_chg &gt; I_charge_allow_bms (vượt trần dòng sạc cho phép của pin).
+• Cờ over_chg_curr từ BMS.
+• Debounce set: 0ms, ngắt STOP tức thì.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
@@ -952,6 +1016,13 @@
           <t>Nhận bản tin ALM_INFO (0x07F4), trường temp_cell_high_dchg. ev_bms() kiểm tra (in-&gt;bms.alarm_flags &amp; BMS_ALARM_TEMP_HIGH_DCHG) != 0.</t>
         </is>
       </c>
+      <c r="H9" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng nhiệt độ xả cao: T_cell &gt;= 60°C khi xả tải.
+• Cờ temp_cell_high_dchg từ BMS.
+• Debounce set: 0ms, cảnh báo INFO.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -989,6 +1060,13 @@
           <t>Nhận bản tin ALM_INFO (0x07F4), trường temp_cell_low_dchg. ev_bms() kiểm tra (in-&gt;bms.alarm_flags &amp; BMS_ALARM_TEMP_LOW_DCHG) != 0.</t>
         </is>
       </c>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng nhiệt độ xả thấp: T_cell &lt; -10°C khi xả tải.
+• Cờ temp_cell_low_dchg từ BMS.
+• Debounce set: 0ms, cảnh báo INFO.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
@@ -1026,6 +1104,13 @@
           <t>Nhận bản tin ALM_INFO (0x07F4), trường temp_relay_high. ev_bms() kiểm tra (in-&gt;bms.alarm_flags &amp; BMS_ALARM_TEMP_RELAY_HIGH) != 0.</t>
         </is>
       </c>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng nhiệt độ MOSFET / Rơ-le: T_relay &gt;= 85°C - 95°C.
+• Cờ temp_relay_high từ BMS.
+• Debounce set: 0ms, cảnh báo INFO.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
@@ -1063,6 +1148,13 @@
           <t>Nhận bản tin ALM_INFO (0x07F4), trường over_dchg_curr. ev_bms() kiểm tra (in-&gt;bms.alarm_flags &amp; BMS_ALARM_OVER_DCHG_CURR) != 0.</t>
         </is>
       </c>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng quá dòng xả: I_dischg &gt; I_discharge_max của khối pin.
+• Cờ over_dchg_curr từ BMS.
+• Debounce set: 0ms, cảnh báo INFO.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
@@ -1100,6 +1192,13 @@
           <t>bms_core.c đếm: now - last_rx_tick &gt; BMS_OFFLINE_TIMEOUT_MS = 5000ms. Quá 5s không nhận được frame nào: gán bms.online = false -&gt; ev_bms_comm_lost() kích hoạt ALARM_BMS_COMM_LOST.</t>
         </is>
       </c>
+      <c r="H13" s="23" t="inlineStr">
+        <is>
+          <t>• Timeout mất CAN BMS: now - last_rx_tick &gt; 5000ms (5.0 giây).
+• Trạng thái áp dụng: BMS_CONTROLLED trong phiên sạc hoạt động.
+• Debounce set: 200ms, clear: 500ms.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="42" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
@@ -1137,6 +1236,13 @@
           <t>BMS online nhưng bms.batt_voltage &lt; cfg_vmax_v * 0.5f. Hàm ev_bms_no_pack_voltage() kích hoạt sau debounce 500ms.</t>
         </is>
       </c>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng nhận diện không pin: Vbatt &lt; 0.5 * Vmax (dưới 50% điện áp định mức).
+• Điều kiện: BMS đang báo online nhưng điện áp cực pin không có.
+• Debounce set: 500ms, clear: 1000ms. Ngắt sạc STOP.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
@@ -1174,6 +1280,15 @@
           <t>Nhận cờ CAN từ bộ sạc: (in-&gt;mod_alarm_or &amp; CHG_LIB_ALARM_HW_FAULT) != 0. Debounce động theo trạng thái: IDLE = 10.000ms (10s) để lọc sạch xung xả tụ/sụt áp khi ngắt Aptomat AC; ACTIVE/RUNNING = 1.000ms (1s) ngắt sạc nhanh an toàn. Tự động suppress khi có sụt áp AC, lỗi PFC, mất pha lưới hoặc khi module offline trong IDLE.</t>
         </is>
       </c>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>• Cờ HW_FAULT (Module fault Byte 7 Bit 1 = 1 từ LianMing / TonHe / Maxwell).
+• Debounce IDLE: 10.000ms (10.0 giây) để lọc sạch 100% quá trình xả tụ (0.2s - 1.5s) khi ngắt Aptomat AC.
+• Debounce ACTIVE (Đang sạc): 1.000ms (1.0 giây) ngắt sạc nhanh.
+• Debounce clear: 200ms.
+• Tự động suppress khi module offline trong IDLE hoặc khi có sụt áp AC/PFC.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
@@ -1211,6 +1326,13 @@
           <t>chg_lib đếm thời gian: now - module[i].last_rx_tick &gt; 2000ms. Quá 2000ms không nhận được phản hồi: gán online = false và bật cờ CHG_LIB_ALARM_COMM_FAIL.</t>
         </is>
       </c>
+      <c r="H16" s="23" t="inlineStr">
+        <is>
+          <t>• Timeout mất CAN module: now - last_rx_tick &gt; 2000ms (2.0 giây).
+• Áp dụng trong RUNNING / READY / PRECHARGE.
+• Debounce set: 0ms, clear: 200ms (ALARM_DB_MODULE_COMM_CLEAR_MS).</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
@@ -1248,6 +1370,13 @@
           <t>Bộ sạc tự phát hiện và gửi qua CAN (Mirror 1:1): Kiểm tra trực tiếp cờ (in-&gt;mod_alarm_or &amp; CHG_LIB_ALARM_OVER_TEMP) != 0.</t>
         </is>
       </c>
+      <c r="H17" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng nhiệt độ tản nhiệt module: T_heatsink &gt;= 85°C - 90°C.
+• Cờ OVER_TEMP từ module sạc.
+• Debounce set: 0ms, clear: 200ms. Ngắt STOP dập dòng an toàn.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
@@ -1285,6 +1414,13 @@
           <t>Bộ sạc tự phát hiện và gửi qua CAN (Mirror 1:1): Kiểm tra cờ (in-&gt;mod_alarm_or &amp; CHG_LIB_ALARM_OVER_VOLTAGE_OUT) != 0.</t>
         </is>
       </c>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng quá áp DC đầu ra: V_out &gt; V_max_hardware của module (thường &gt; 750V hoặc &gt; 1000V).
+• Cờ OVER_VOLTAGE_OUT từ module.
+• Debounce set: 0ms, ngắt ESTOP tức thì mở relay.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="42" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
@@ -1322,6 +1458,13 @@
           <t>Bộ sạc tự phát hiện và gửi qua CAN (Mirror 1:1): Kiểm tra cờ (in-&gt;mod_alarm_or &amp; CHG_LIB_ALARM_SHORT_CIRCUIT) != 0.</t>
         </is>
       </c>
+      <c r="H19" s="23" t="inlineStr">
+        <is>
+          <t>• Ngắn mạch đầu ra: Điện trở tải R_load ~ 0 Ohm, V_out sập về 0V khi đang phát dòng.
+• Cờ SHORT_CIRCUIT từ module (bảo vệ ngắt xung phần cứng &lt; 10us).
+• Debounce set: 0ms, ngắt ESTOP tức thì mở relay.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="42" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
@@ -1359,6 +1502,13 @@
           <t>Bộ sạc tự phát hiện và gửi qua CAN (Mirror 1:1): Kiểm tra cờ (in-&gt;mod_alarm_or &amp; CHG_LIB_ALARM_OVER_CURR_OUT) != 0.</t>
         </is>
       </c>
+      <c r="H20" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng quá dòng đầu ra: I_out &gt; 110% dòng định mức module (ví dụ module 50A ngắt khi I &gt; 55A).
+• Cờ OVER_CURR_OUT từ module.
+• Debounce set: 0ms, clear: 200ms. Ngắt STOP.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
@@ -1396,6 +1546,13 @@
           <t>Nhận cờ CAN lỗi PFC/mất pha từ bộ sạc: ev_mod_pfc kích hoạt. Tự động bypass ở IDLE (chống báo ảo khi ngắt AC), suppress khi có cờ thấp áp AC.</t>
         </is>
       </c>
+      <c r="H21" s="23" t="inlineStr">
+        <is>
+          <t>• Lỗi tầng chỉnh lưu PFC: Mất pha, quá áp/thấp áp bus nội bộ PFC.
+• Ở IDLE: Tự động BYPASS hoàn toàn.
+• Ở ACTIVE: Debounce set: 0ms, clear: 200ms. Suppress khi có sụt áp AC.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
@@ -1433,6 +1590,13 @@
           <t>Bộ sạc tự phát hiện và gửi qua CAN (Mirror 1:1): Kiểm tra trực tiếp cờ (in-&gt;mod_alarm_or &amp; CHG_LIB_ALARM_FAN_FAULT) != 0.</t>
         </is>
       </c>
+      <c r="H22" s="23" t="inlineStr">
+        <is>
+          <t>• Lỗi quạt tản nhiệt: Tốc độ quạt &lt; 500 RPM khi module đang chạy, hoặc đứt dây feedback FG.
+• Cờ FAN_FAULT từ module.
+• Debounce set: 0ms, clear: 200ms. Ngắt STOP.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="42" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
@@ -1470,6 +1634,13 @@
           <t>Bộ sạc tự phát hiện và gửi qua CAN (Mirror 1:1): Kiểm tra trực tiếp cờ (in-&gt;mod_alarm_or &amp; CHG_LIB_ALARM_AC_OVER_VOLT) != 0.</t>
         </is>
       </c>
+      <c r="H23" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng quá áp lưới AC 3 pha: V_dây (V_line-line) &gt; 456 VAC - 475 VAC (tương đương V_pha &gt; 263 VAC - 274 VAC).
+• Cờ AC_OVER_VOLT từ module.
+• Debounce set: 0ms, clear: 200ms. Ngắt STOP.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="42" customHeight="1">
       <c r="A24" s="7" t="inlineStr">
@@ -1507,6 +1678,14 @@
           <t>Nhận cờ CAN thấp áp AC: (in-&gt;mod_alarm_or &amp; CHG_LIB_ALARM_AC_UNDER_VOLT) != 0. Tự động bypass trong IDLE (Clean Shutdown); trong active session debounce set 1000ms, clear 3000ms.</t>
         </is>
       </c>
+      <c r="H24" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng thấp áp lưới AC 3 pha: V_dây (V_line-line) &lt; 280 VAC - 300 VAC (tương đương V_pha &lt; 160 VAC - 173 VAC).
+• Ở IDLE: Tự động BYPASS hoàn toàn (Clean Shutdown khi ngắt CB).
+• Ở ACTIVE: Debounce set: 1000ms (1.0s), clear: 3000ms (3.0s).
+• Chế áp E010, E015, W010.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="42" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
@@ -1544,6 +1723,14 @@
           <t>ev_dc_load_lost() trong alarm.c: Đang RUNNING và dòng sụt &lt; 15% dòng đặt mục tiêu trong khi áp &gt; 98% áp mục tiêu. Debounce: 800ms. Latching = true.</t>
         </is>
       </c>
+      <c r="H25" s="23" t="inlineStr">
+        <is>
+          <t>• Điều kiện mất tải DC (Hot Unplug): Dòng sụt I &lt; 15% dòng đặt (ALARM_LOAD_LOST_I_FRAC = 0.15) trong khi áp V &gt; 98% áp đặt (ALARM_V_AT_TARGET_FRAC = 0.98).
+• Điều kiện dòng đặt: I_applied &gt;= 2.0A (ALARM_I_LOAD_MIN_A).
+• Debounce set: 800ms (ALARM_LOAD_LOST_MS).
+• Chốt giữ mã lỗi (Latching = true), clear delay: 3000ms.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="42" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
@@ -1581,6 +1768,13 @@
           <t>ev_dc_out_not_established() trong alarm.c: Đã phát lệnh đóng rơ-le quá 5000ms nhưng dòng sạc đo được vẫn &lt; 2.0A. Latching = true.</t>
         </is>
       </c>
+      <c r="H26" s="23" t="inlineStr">
+        <is>
+          <t>• Thời gian chờ hình thành dòng: Sau lệnh đóng relay 12000ms (12.0 giây, ALARM_DC_OUT_CONFIRM_MS).
+• Ngưỡng dòng xác nhận: Tổng dòng sạc I_total &lt; 2.0A (ALARM_I_LOAD_MIN_A).
+• Chốt giữ mã lỗi (Latching = true), clear delay: 3000ms.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="42" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
@@ -1618,6 +1812,12 @@
           <t>Khi nhận lệnh sạc, charge_controller.c kiểm tra mod_online_count == 0 hoặc driver chưa chọn -&gt; cờ CHARGE_CTRL_FAULT_NO_MODULE.</t>
         </is>
       </c>
+      <c r="H27" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng module: Số module sạc online thực tế = 0 (actual_count == 0).
+• Kích hoạt tại thời điểm bắt đầu khởi động sạc.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="42" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
@@ -1655,6 +1855,12 @@
           <t>actual_module_count != configured_module_count -&gt; cờ CHARGE_CTRL_FAULT_MODULE_COUNT_MISMATCH -&gt; ALARM_CTRL_MODULE_MISMATCH.</t>
         </is>
       </c>
+      <c r="H28" s="23" t="inlineStr">
+        <is>
+          <t>• Sai lệch số module: actual_count != cfg.source_module_count (ví dụ cấu hình 2 module nhưng chỉ có 1 module online).
+• Từ chối sạc (Inhibit).</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="42" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
@@ -1692,6 +1898,12 @@
           <t>ChargeCycleConfig_Set() từ chối cấu hình -&gt; cờ CHARGE_CTRL_FAULT_INVALID_CONFIG -&gt; ALARM_CTRL_INVALID_CONFIG.</t>
         </is>
       </c>
+      <c r="H29" s="23" t="inlineStr">
+        <is>
+          <t>• Lỗi cấu hình: cfg.version != 9 hoặc Vmax &lt;= Vmin hoặc Imax &lt;= 0.
+• Từ chối sạc (Inhibit).</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="42" customHeight="1">
       <c r="A30" s="7" t="inlineStr">
@@ -1729,6 +1941,14 @@
           <t>So sánh |Volt_target - Volt_max| &gt; 2.0V, trong đó Volt_target lấy từ bản tin CAN BMS ChgRequest_INFO (0x1806E5F4) và Volt_max lấy theo cấu hình cài đặt sạc (cfg.vmax_v). Debounce 1000ms. ev_bms_volt_mismatch() kích hoạt ALARM_BMS_VOLT_MISMATCH.</t>
         </is>
       </c>
+      <c r="H30" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng sai lệch điện áp cắm sạc: |V_target_bms - V_max_cfg| &gt; 2.0V.
+• Điều kiện: V_target_bms &gt; 10.0V và V_max_cfg &gt; 10.0V.
+• Debounce set: 1000ms (1.0s), clear: 500ms.
+• Ngắt STOP chống cắm nhầm sạc.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="42" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
@@ -1766,6 +1986,14 @@
           <t>V_module - V_bms vượt ngưỡng threshold cấu hình trong khoảng thời gian trip delay -&gt; CHARGE_CTRL_FAULT_PROTECT_JACK_V.</t>
         </is>
       </c>
+      <c r="H31" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng sụt áp tiếp xúc jack: Delta_V = (V_module - V_bms) &gt; 2.0V (protect_jack_charge_delta_v, dải 0.5V - 10.0V).
+• Điều kiện dòng: I_total &gt;= 2.0A và relay đã chốt đóng.
+• Thời gian trễ xác nhận: Duy trì liên tục &gt;= 3.0 giây (protect_jack_charge_delay_s).
+• Gián đoạn bất kỳ tick nào sẽ tự động reset timer về 0.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="42" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
@@ -1801,6 +2029,13 @@
       <c r="G32" s="8" t="inlineStr">
         <is>
           <t>Cảm biến nhiệt độ NTC jack sạc vượt ngưỡng cấu hình -&gt; CHARGE_CTRL_FAULT_PROTECT_JACK_TEMP.</t>
+        </is>
+      </c>
+      <c r="H32" s="23" t="inlineStr">
+        <is>
+          <t>• Ngưỡng ngắt sạc quá nhiệt jack: T_jack &gt;= 70°C - 80°C (protect_jack_temp_trip_c) đo từ 4 cảm biến NTC (PA0..PA3).
+• Ngưỡng cảnh báo / giảm dòng (Derating): T_jack &gt;= 60°C (protect_jack_temp_warn_c).
+• Ngắt STOP khẩn cấp khi vượt ngưỡng trip.</t>
         </is>
       </c>
     </row>
@@ -1978,7 +2213,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
@@ -2121,7 +2355,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
         <is>
@@ -2291,7 +2524,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
         <is>
@@ -2555,7 +2787,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(charge): implement fault-tolerant parallel charging, dynamic load rebalancing, and bump to V2.0.19
</commit_message>
<xml_diff>
--- a/docs/BANG_MA_LOI_HE_THONG.xlsx
+++ b/docs/BANG_MA_LOI_HE_THONG.xlsx
@@ -1267,12 +1267,12 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Dừng sạc an toàn (STOP)</t>
+          <t>Cảnh báo (INFO / Degraded) nếu còn &gt;= 1 module; Dừng sạc (STOP) nếu hỏng toàn bộ</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>Bộ sạc tự phát hiện hỏng hóc linh kiện công suất: Hỏng nguồn nuôi phụ cấp (+15V, +5V, -15V), rơ-le xả mềm bị dính/hỏng, lỗi cảm biến hoặc EEPROM.</t>
+          <t>Bộ sạc tự phát hiện hỏng hóc linh kiện công suất: Hỏng nguồn nuôi phụ cấp (+15V, +5V, -15V), rơ-le xả mềm bị dính/hỏng, lỗi cảm biến hoặc EEPROM. Trong hệ thống đa module: nếu còn ít nhất 1 module hoạt động bình thường, hạ cấp về INFO, loại module lỗi ra, tự động san tải cho các module còn lại và tiếp tục sạc. Chỉ ngắt STOP khi toàn bộ module đều hỏng.</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Dừng sạc an toàn (STOP)</t>
+          <t>Cảnh báo (INFO / Degraded) nếu còn &gt;= 1 module; Dừng sạc (STOP) nếu hỏng toàn bộ</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>Nhiệt độ khối tản nhiệt (Heatsink) hoặc biến áp xung DC-DC bên trong bộ sạc vượt quá ngưỡng cho phép (thường &gt; 85°C - 90°C).</t>
+          <t>Nhiệt độ khối tản nhiệt (Heatsink) hoặc biến áp xung DC-DC bên trong bộ sạc vượt quá ngưỡng cho phép (thường &gt; 85°C - 90°C). Trong hệ thống đa module: tự động hạ cấp về INFO khi còn &gt;= 1 module lành.</t>
         </is>
       </c>
       <c r="G17" s="12" t="inlineStr">
@@ -1489,12 +1489,12 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Dừng sạc an toàn (STOP)</t>
+          <t>Cảnh báo (INFO / Degraded) nếu còn &gt;= 1 module; Dừng sạc (STOP) nếu hỏng toàn bộ</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>Dòng điện thực tế ngõ ra của bộ sạc vượt quá ngưỡng dòng điện định mức tối đa (I &gt; 110% Imax).</t>
+          <t>Dòng điện thực tế ngõ ra của bộ sạc vượt quá ngưỡng dòng điện định mức tối đa (I &gt; 110% Imax). Trong hệ thống đa module: tự động hạ cấp về INFO khi còn &gt;= 1 module lành.</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
@@ -1533,12 +1533,12 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Dừng sạc an toàn (STOP)</t>
+          <t>Cảnh báo (INFO / Degraded) nếu còn &gt;= 1 module; Dừng sạc (STOP) nếu hỏng toàn bộ</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr">
         <is>
-          <t>Khối mạch chỉnh lưu công suất nguồn đầu vào (PFC) của bộ sạc bị sự cố.</t>
+          <t>Khối mạch chỉnh lưu công suất nguồn đầu vào (PFC) của bộ sạc bị sự cố. Trong hệ thống đa module: tự động hạ cấp về INFO khi còn &gt;= 1 module lành.</t>
         </is>
       </c>
       <c r="G21" s="12" t="inlineStr">
@@ -1577,12 +1577,12 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>Dừng sạc an toàn (STOP)</t>
+          <t>Cảnh báo (INFO / Degraded) nếu còn &gt;= 1 module; Dừng sạc (STOP) nếu hỏng toàn bộ</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>Một hoặc nhiều quạt làm mát bên trong bộ sạc bị kẹt cơ học, đứt dây tín hiệu hồi tiếp tốc độ hoặc cháy cuộn dây.</t>
+          <t>Một hoặc nhiều quạt làm mát bên trong bộ sạc bị kẹt cơ học, đứt dây tín hiệu hồi tiếp tốc độ hoặc cháy cuộn dây. Trong hệ thống đa module: tự động hạ cấp về INFO khi còn &gt;= 1 module lành.</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
@@ -1621,12 +1621,12 @@
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Dừng sạc an toàn (STOP)</t>
+          <t>Cảnh báo (INFO / Degraded) nếu còn &gt;= 1 module; Dừng sạc (STOP) nếu hỏng toàn bộ</t>
         </is>
       </c>
       <c r="F23" s="12" t="inlineStr">
         <is>
-          <t>Điện áp lưới điện AC 3 pha vượt quá ngưỡng bảo vệ tối đa của bộ sạc (thường &gt; 456 VAC).</t>
+          <t>Điện áp lưới điện AC 3 pha vượt quá ngưỡng bảo vệ tối đa của bộ sạc (thường &gt; 456 VAC). Trong hệ thống đa module: tự động hạ cấp về INFO khi còn &gt;= 1 module lành.</t>
         </is>
       </c>
       <c r="G23" s="12" t="inlineStr">
@@ -1799,23 +1799,23 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Từ chối sạc (Inhibit)</t>
+          <t>Dừng sạc an toàn (STOP) / Từ chối sạc</t>
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr">
         <is>
-          <t>Bo điều khiển trung tâm quét trên đường truyền CAN nhưng không phát hiện được bất kỳ bộ sạc nào phản hồi online tại thời điểm khởi tạo hệ thống.</t>
+          <t>Bộ điều khiển trung tâm không phát hiện được bất kỳ bộ sạc nào phản hồi online tại thời điểm khởi tạo, HOẶC toàn bộ module online bị mất (N_actual == 0) kéo dài quá debounce 10s trong lúc đang sạc.</t>
         </is>
       </c>
       <c r="G27" s="12" t="inlineStr">
         <is>
-          <t>Khi nhận lệnh sạc, charge_controller.c kiểm tra mod_online_count == 0 hoặc driver chưa chọn -&gt; cờ CHARGE_CTRL_FAULT_NO_MODULE.</t>
+          <t>mod_online_count == 0 -&gt; CHARGE_CTRL_FAULT_NO_MODULE. Khi đang sạc: timer debounce 10s mất hết module -&gt; kích hoạt ngắt STOP an toàn.</t>
         </is>
       </c>
       <c r="H27" s="23" t="inlineStr">
         <is>
-          <t>• Ngưỡng module: Số module sạc online thực tế = 0 (actual_count == 0).
-• Kích hoạt tại thời điểm bắt đầu khởi động sạc.</t>
+          <t>• Khởi động: N_actual == 0 -&gt; Từ chối sạc (Inhibit).
+• Đang sạc: N_actual == 0 duy trì liên tục quá 10.000ms (10s) -&gt; Ngắt an toàn STOP.</t>
         </is>
       </c>
     </row>
@@ -1842,23 +1842,24 @@
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>Từ chối sạc (Inhibit)</t>
+          <t>Cảnh báo (INFO / Degraded)</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>Số lượng bộ sạc online thực tế khác với số lượng bộ sạc được thiết lập trong cấu hình hệ thống.</t>
+          <t>Số lượng bộ sạc online thực tế nhỏ hơn số lượng bộ sạc được thiết lập trong cấu hình hệ thống (N_actual &lt; N_source) nhưng vẫn còn ít nhất 1 module hoạt động bình thường.</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>actual_module_count != configured_module_count -&gt; cờ CHARGE_CTRL_FAULT_MODULE_COUNT_MISMATCH -&gt; ALARM_CTRL_MODULE_MISMATCH.</t>
+          <t>actual_module_count &lt; configured_module_count -&gt; cờ CHARGE_CTRL_FAULT_MODULE_COUNT_MISMATCH -&gt; ALARM_CTRL_MODULE_MISMATCH (action INFO). Tự động suppress khi có W010 (mất CAN) hoặc W011 (sụt áp AC).</t>
         </is>
       </c>
       <c r="H28" s="23" t="inlineStr">
         <is>
-          <t>• Sai lệch số module: actual_count != cfg.source_module_count (ví dụ cấu hình 2 module nhưng chỉ có 1 module online).
-• Từ chối sạc (Inhibit).</t>
+          <t>• Sai lệch: N_actual &lt; cfg.source_module_count (khi N_actual &gt;= 1).
+• Vẫn tiếp tục sạc ở chế độ dự phòng (Degraded Mode), tự động chia lại tải I_target / N_actual và kẹp trần công suất theo N_actual * I_max_mod.
+• Cảnh báo INFO trên DWIN/PC App.</t>
         </is>
       </c>
     </row>
@@ -2130,7 +2131,8 @@
 2. Gửi lệnh giảm dòng mục tiêu target_current = 0A qua mạng CAN tới tất cả module.
 3. Chờ dòng điện phản hồi thực tế giảm xuống &lt; 1.0A (RELAY_OPEN_CURRENT_THRESHOLD_A) để dập hồ quang (hoặc timeout 3000ms).
 4. Mở rơ-le / contactor DC ngõ ra sạc.
-5. Ghi log sự kiện vào RAM Ring Buffer (sâu 16 bản ghi) và lưu trữ vĩnh viễn vào External SPI Flash (W25Qxx).</t>
+5. Ghi log sự kiện vào RAM Ring Buffer (sâu 16 bản ghi) và lưu trữ vĩnh viễn vào External SPI Flash (W25Qxx).
+* Áp dụng cho các lỗi module cục bộ (E010, E011, E014..E017) khi TOÀN BỘ module đều hỏng (N_actual = 0).</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2182,8 @@
           <t>1. Không ngắt chu trình sạc hiện tại.
 2. Bật bit trạng thái trong AlarmView_t.active_mask.
 3. Gửi mã cảnh báo và chuỗi UTF-16 hiển thị màu vàng trên màn hình DWIN HMI và app PC.
-4. Tự động xóa cảnh báo khi điều kiện vật lý trở lại bình thường qua thời gian debounce.</t>
+4. Tự động xóa cảnh báo khi điều kiện vật lý trở lại bình thường qua thời gian debounce.
+* Bao gồm E028 và các lỗi module cục bộ (E010, E011, E014..E017) khi còn &gt;= 1 module lành để duy trì sạc suy giảm (Degraded Mode).</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="65" customWidth="1" min="1" max="1"/>
@@ -2956,6 +2959,60 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Mất CAN bộ sạc hoặc Sụt áp AC (W010 / W011)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>W010 hoặc W011</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>E028 (Số bộ sạc không khớp)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>ev_ctrl_module_mismatch() kiểm tra cờ W010 và W011 active/latched -&gt; suppress E028 hoàn toàn.</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Tránh báo đè lỗi số lượng khi nguyên nhân cốt lõi là do mất kết nối CAN hoặc mất pha AC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Lỗi cục bộ 1 module trong hệ thống đa module</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>E010, E011, E014, E015, E016, E017 (Cảnh báo INFO)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Dừng sạc toàn trạm (STOP Action)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>get_effective_action() hạ cấp hành vi lỗi module từ STOP xuống INFO khi N_active &gt;= 1; chỉ nâng lên STOP khi N_active == 0.</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Duy trì sạc liên tục ở chế độ suy giảm (Fault-Tolerant Degraded Charging), tự động tái cân bằng tải.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(excel): update BANG_MA_LOI_HE_THONG.xlsx with V2.0.22 per-module alarm specifications
</commit_message>
<xml_diff>
--- a/docs/BANG_MA_LOI_HE_THONG.xlsx
+++ b/docs/BANG_MA_LOI_HE_THONG.xlsx
@@ -1267,7 +1267,7 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Cảnh báo (INFO / Degraded) nếu còn &gt;= 1 module; Dừng sạc (STOP) nếu hỏng toàn bộ</t>
+          <t>Trạm 1 module: Dừng sạc an toàn (STOP), text chuẩn không [M1]. Trạm đa module (N &gt;= 2): Cảnh báo (INFO / Degraded) hiển thị đích danh [M1]..[M8] nếu còn &gt;= 1 module tốt; STOP nếu hỏng hết.</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Cảnh báo (INFO) nếu mất 1 phần; Dừng sạc (STOP) nếu mất hết</t>
+          <t>Trạm 1 module: Dừng sạc an toàn (STOP), text chuẩn không [M1]. Trạm đa module (N &gt;= 2): Cảnh báo (INFO / Degraded) hiển thị đích danh [M1]..[M8] nếu còn &gt;= 1 module tốt; STOP nếu hỏng hết.</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Cảnh báo (INFO / Degraded) nếu còn &gt;= 1 module; Dừng sạc (STOP) nếu hỏng toàn bộ</t>
+          <t>Trạm 1 module: Dừng sạc an toàn (STOP), text chuẩn không [M1]. Trạm đa module (N &gt;= 2): Cảnh báo (INFO / Degraded) hiển thị đích danh [M1]..[M8] nếu còn &gt;= 1 module tốt; STOP nếu hỏng hết.</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Cảnh báo (INFO / Degraded) nếu còn &gt;= 1 module; Dừng sạc (STOP) nếu hỏng toàn bộ</t>
+          <t>Trạm 1 module: Dừng sạc an toàn (STOP), text chuẩn không [M1]. Trạm đa module (N &gt;= 2): Cảnh báo (INFO / Degraded) hiển thị đích danh [M1]..[M8] nếu còn &gt;= 1 module tốt; STOP nếu hỏng hết.</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Cảnh báo (INFO / Degraded) nếu còn &gt;= 1 module; Dừng sạc (STOP) nếu hỏng toàn bộ</t>
+          <t>Trạm 1 module: Dừng sạc an toàn (STOP), text chuẩn không [M1]. Trạm đa module (N &gt;= 2): Cảnh báo (INFO / Degraded) hiển thị đích danh [M1]..[M8] nếu còn &gt;= 1 module tốt; STOP nếu hỏng hết.</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>Cảnh báo (INFO / Degraded) nếu còn &gt;= 1 module; Dừng sạc (STOP) nếu hỏng toàn bộ</t>
+          <t>Trạm 1 module: Dừng sạc an toàn (STOP), text chuẩn không [M1]. Trạm đa module (N &gt;= 2): Cảnh báo (INFO / Degraded) hiển thị đích danh [M1]..[M8] nếu còn &gt;= 1 module tốt; STOP nếu hỏng hết.</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Cảnh báo (INFO / Degraded) nếu còn &gt;= 1 module; Dừng sạc (STOP) nếu hỏng toàn bộ</t>
+          <t>Trạm 1 module: Dừng sạc an toàn (STOP), text chuẩn không [M1]. Trạm đa module (N &gt;= 2): Cảnh báo (INFO / Degraded) hiển thị đích danh [M1]..[M8] nếu còn &gt;= 1 module tốt; STOP nếu hỏng hết.</t>
         </is>
       </c>
       <c r="F23" s="12" t="inlineStr">
@@ -2198,7 +2198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="65" customWidth="1" min="1" max="1"/>
@@ -2437,12 +2437,12 @@
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>0 .. 65535 (AlarmCode_t)</t>
+          <t>Mã 16-bit (Bit 0..7: Code, Bit 8..15: Source ID)</t>
         </is>
       </c>
       <c r="E13" s="19" t="inlineStr">
         <is>
-          <t>Mã định danh lỗi: ánh xạ trực tiếp sang E001..E032, W001..W011.</t>
+          <t>Mã nén 16-bit. Bit 0..7: Mã định danh lỗi (E001..E032, W001..W011). Bit 8..15: Nguồn gốc lỗi (0 = Trạm/BMS/Hệ thống hoặc Trạm đơn 1 module hiển thị nguyên bản; 1..8 = Module 1 đến Module 8 khi trạm chạy song song đa module, HMI DWIN tự động nối hậu tố [M1]..[M8]).</t>
         </is>
       </c>
     </row>
@@ -3010,6 +3010,33 @@
       <c r="E36" t="inlineStr">
         <is>
           <t>Duy trì sạc liên tục ở chế độ suy giảm (Fault-Tolerant Degraded Charging), tự động tái cân bằng tải.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Phân định Trạm đơn (1 module) vs Trạm song song đa module (N &gt;= 2)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Trạm 1 module: Báo lỗi chuẩn không [M1]; Trạm đa module: Báo đích danh [M1]..[M8]</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Hậu tố [M1] trên trạm 1 module; Hành vi dừng trạm khi còn module tốt</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Khi mod_total_count == 1: source_id = 0, DWIN hiển thị text nguyên bản không [M1], lỗi module dừng STOP/ESTOP ngay lập tức (N_active=0). Khi mod_total_count &gt; 1: source_id = m+1, DWIN thêm [M1]..[M8], giáng cấp INFO và duy trì sạc Degraded Mode khi N_active &gt;= 1.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Trạm 1 module báo lỗi tự nhiên và dừng sạc chuẩn mực; trạm đa module chỉ định chính xác module hỏng và không ngắt sạc vô cớ.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(release): Release V2.0.23 - dynamic bidirectional battery voltage mismatch E032 and storage charging support
</commit_message>
<xml_diff>
--- a/docs/BANG_MA_LOI_HE_THONG.xlsx
+++ b/docs/BANG_MA_LOI_HE_THONG.xlsx
@@ -1934,20 +1934,22 @@
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>Khách hàng cắm nhầm chủng loại pin vào máy sạc (ví dụ cắm pin 48V vào sạc 72V hoặc ngược lại).</t>
+          <t>Người vận hành cắm nhầm hệ pin khác với cấu hình bộ sạc (VD: sạc 48V cắm vào pin 72V, hoặc tủ cấu hình 72V cắm vào pack 48V).</t>
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>So sánh |Volt_target - Volt_max| &gt; 2.0V, trong đó Volt_target lấy từ bản tin CAN BMS ChgRequest_INFO (0x1806E5F4) và Volt_max lấy theo cấu hình cài đặt sạc (cfg.vmax_v). Debounce 1000ms. ev_bms_volt_mismatch() kích hoạt ALARM_BMS_VOLT_MISMATCH.</t>
+          <t>So sánh độ lệch điện áp 2 chiều giữa cấu hình sạc (Vmax) và yêu cầu từ BMS (Vtarget) hoặc điện áp thực tế cọc bình (Vbatt) với ngưỡng động delta_V_thresh = max(10.0V, 16% * Vmax). Debounce: 1000ms.</t>
         </is>
       </c>
       <c r="H30" s="23" t="inlineStr">
         <is>
-          <t>• Ngưỡng sai lệch điện áp cắm sạc: |V_target_bms - V_max_cfg| &gt; 2.0V.
-• Điều kiện: V_target_bms &gt; 10.0V và V_max_cfg &gt; 10.0V.
+          <t>• Ngưỡng sai lệch hệ pin động: delta_V_thresh = max(10.0V, 16% * Vmax_cfg).
+• Báo lỗi khi |Vtarget_bms - Vmax_cfg| &gt;= delta_V_thresh HOẶC (Vbatt - Vmax_cfg) &gt;= delta_V_thresh (chống xả ngược).
+• Tự động co giãn theo cấp điện áp: Hệ 12V-48V áp dụng sàn cứng 10V (khách cài 50V sạc lưu kho 50% SOC pack 16S LFP không bị lỗi); hệ cao áp 72V-500V tự động nới theo tỷ lệ 16% bảo vệ chống nhầm hệ pin.
+• Điều kiện: Chế độ BMS Controlled, Vmax_cfg &gt; 10.0V.
 • Debounce set: 1000ms (1.0s), clear: 500ms.
-• Ngắt STOP chống cắm nhầm sạc.</t>
+• Ngắt STOP an toàn, bảo vệ cả pin và tủ sạc.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(release): Release V2.0.24 - senior bidirectional volt mismatch E032 with instant hardware back-feed protection
</commit_message>
<xml_diff>
--- a/docs/BANG_MA_LOI_HE_THONG.xlsx
+++ b/docs/BANG_MA_LOI_HE_THONG.xlsx
@@ -1939,17 +1939,17 @@
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>So sánh độ lệch điện áp 2 chiều giữa cấu hình sạc (Vmax) và yêu cầu từ BMS (Vtarget) hoặc điện áp thực tế cọc bình (Vbatt) với ngưỡng động delta_V_thresh = max(10.0V, 16% * Vmax). Debounce: 1000ms.</t>
+          <t>Thuật toán xét 2 chiều độc lập: 1) Bảo vệ phần cứng tức thời chống xả ngược: Vbatt &gt; Vmax + 2.0V; 2) Tách biệt danh định bất đối xứng: Sạc lớn cắm pin nhỏ: Vmax - Vreq &gt;= max(12V, 18%*Vmax); Sạc nhỏ cắm pin lớn khi cạn: Vreq - Vmax &gt;= max(10V, 15%*Vmax). Debounce: 1000ms.</t>
         </is>
       </c>
       <c r="H30" s="23" t="inlineStr">
         <is>
-          <t>• Ngưỡng sai lệch hệ pin động: delta_V_thresh = max(10.0V, 16% * Vmax_cfg).
-• Báo lỗi khi |Vtarget_bms - Vmax_cfg| &gt;= delta_V_thresh HOẶC (Vbatt - Vmax_cfg) &gt;= delta_V_thresh (chống xả ngược).
-• Tự động co giãn theo cấp điện áp: Hệ 12V-48V áp dụng sàn cứng 10V (khách cài 50V sạc lưu kho 50% SOC pack 16S LFP không bị lỗi); hệ cao áp 72V-500V tự động nới theo tỷ lệ 16% bảo vệ chống nhầm hệ pin.
-• Điều kiện: Chế độ BMS Controlled, Vmax_cfg &gt; 10.0V.
-• Debounce set: 1000ms (1.0s), clear: 500ms.
-• Ngắt STOP an toàn, bảo vệ cả pin và tủ sạc.</t>
+          <t>• Bảo vệ phần cứng tức thời: Vbatt &gt; Vmax + 2.0V kích hoạt ngay lập tức.
+• Tách biệt 2 chiều bất đối xứng:
+  + Sạc lớn cắm pin nhỏ: Vmax - Vreq &gt;= max(12V, 18%*Vmax)
+  + Sạc nhỏ cắm pin lớn: Vreq - Vmax &gt;= max(10V, 15%*Vmax)
+• Hỗ trợ sạc bảo quản / non tải (cài 113V sạc pin 32S 112V bình thường).
+• Debounce set: 1000ms, clear: 500ms.</t>
         </is>
       </c>
     </row>

</xml_diff>